<commit_message>
match spreadsheet local authority with that expected
</commit_message>
<xml_diff>
--- a/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
+++ b/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sprior\source\repos\rsd-lsrp-validation-function\src\Tests\GovUK.Dfe.Lsrp.FileValidator.Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19117182-89D2-47F9-A261-F9C833B9B348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD30C2D8-77A0-400A-9C16-48FC0441162C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="54615" yWindow="6180" windowWidth="16050" windowHeight="9405" activeTab="2" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
+    <workbookView xWindow="34440" yWindow="-4590" windowWidth="38640" windowHeight="21120" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="2" r:id="rId1"/>
@@ -41,12 +41,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>2026-27 Data</t>
   </si>
   <si>
     <t>The Local SEND Reform Plan</t>
+  </si>
+  <si>
+    <t>LA1</t>
   </si>
 </sst>
 </file>
@@ -418,9 +421,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C342540-87D2-434A-ACBB-5DDA8DCA1D3F}">
-  <dimension ref="A1"/>
+  <dimension ref="B13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Spreadsheet validation now handles local authority check (#8)
* match spreadsheet local authority with that expected

* refactor validation function to improve design

* change function log error to log info

---------

Co-authored-by: PRIOR <Stephen.PRIOR@EDUCATION.GOV.UK>
</commit_message>
<xml_diff>
--- a/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
+++ b/src/Tests/GovUK.Dfe.Lsrp.FileValidator.Tests/qr-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sprior\source\repos\rsd-lsrp-validation-function\src\Tests\GovUK.Dfe.Lsrp.FileValidator.Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19117182-89D2-47F9-A261-F9C833B9B348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD30C2D8-77A0-400A-9C16-48FC0441162C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="54615" yWindow="6180" windowWidth="16050" windowHeight="9405" activeTab="2" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
+    <workbookView xWindow="34440" yWindow="-4590" windowWidth="38640" windowHeight="21120" xr2:uid="{6BD4A847-062F-4B04-BCC0-51F7CFC614FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="2" r:id="rId1"/>
@@ -41,12 +41,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>2026-27 Data</t>
   </si>
   <si>
     <t>The Local SEND Reform Plan</t>
+  </si>
+  <si>
+    <t>LA1</t>
   </si>
 </sst>
 </file>
@@ -418,9 +421,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C342540-87D2-434A-ACBB-5DDA8DCA1D3F}">
-  <dimension ref="A1"/>
+  <dimension ref="B13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>